<commit_message>
Simplify tract gallery deployment
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tracts.xlsx
+++ b/tracts.xlsx
@@ -545,160 +545,160 @@
     <t>Bilans des accords signés par la CGT_page-0001.jpg</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Tract-retraites-2026-v-allegee.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/communaut%C3%A9%20whatsapp%20v2.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/2026_06_TRACT-RetourSondageRCC2026-2.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/repression%20syndicale%20v5.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract_perform_to_win.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract_pour_ceux_qui_restent.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Soutien_Grece_Nokia_Microwave_v1.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract_rcc_2026.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract%20evaluation%20objectifs%20v2--3p.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract%20AT.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/reponse%20gaza%202025%20v4.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/20250827_Mobilisation_10_Septembre_CCN.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract%20contentieux%20bonus%2016juin25.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract_palestine_appel_manif.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/20250507_JourneeAction5Juin_Tract_.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/2025_04_TRACT_radar_restitution_v2_3p.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract-salaires-2025.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract-prevention-risques_V1.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract-avenant-TL-v2.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract_calculateur_salaires_2025.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/CGT-NPS-Voeux-2025.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract-indus-v1.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/2024-12-04_Mobilisations_et_elections_TPE.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract_bilan_rcc24_v4.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract_democratie_rcc_salaires_v2.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Profession_de_Foi_CGT_elections_FCPAN_2024_VF_V3.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract_retour_salaires_2024_v1.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/reorg-mn-V3.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract-noel-2023-V3.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/ncc%20cotation%203.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract_annonces_pekka_06_11_2023.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract_militants_nord.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/tract%20com%20nokia%20final.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/midpoints.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Tract%20Volontariat%20RCC.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Tract%20br%C3%A8ves%20de%20printemps.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Tract_Sant%C3%A9_Pr%C3%A9voyance_Mars_2022%20nps.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Tract%20CGT%20desaccords%20en%20cascade%2003-06-2022.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Tract%20br%C3%A8ves%20d%27%C3%A9t%C3%A9.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Tract%20demenagement%2006-09-22.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Manif29septembre%20CandidaturesElection.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Ce%20que%20veulent%20les%20Cadres%20-Synth%C3%A8se%20Barom%C3%A8tre%20Cadres%20UGICT%20Viavoice%20octobre%202022.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Retour%20Sondage%20CGT%20Navettes%20Octobre%202022.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Les%20Navettes%20Quelle%20Gal%C3%A8re%2009_11_2022.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Radar%20Travail%20et%20Environnement%2009_11_2022.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Le%20saviez-vous%2012_11_2022.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Points%20sur%20les%20i%2012_11_2022.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Elections%20Pro%20-%20Choisir%20son%20camp.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Enjeu%20Salaires2022.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Tract%20Sondages.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Tract_NegoTELEW.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/copies/Bilans%20des%20accords%20sign%C3%A9s%20par%20la%20CGT.pdf</t>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Tract-retraites-2026-v-allegee.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/communaut%C3%A9%20whatsapp%20v2.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/2026_06_TRACT-RetourSondageRCC2026-2.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/repression%20syndicale%20v5.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_perform_to_win.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_pour_ceux_qui_restent.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Soutien_Grece_Nokia_Microwave_v1.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_rcc_2026.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract%20evaluation%20objectifs%20v2--3p.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract%20AT.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/reponse%20gaza%202025%20v4.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/20250827_Mobilisation_10_Septembre_CCN.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract%20contentieux%20bonus%2016juin25.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_palestine_appel_manif.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/20250507_JourneeAction5Juin_Tract_.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/2025_04_TRACT_radar_restitution_v2_3p.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract-salaires-2025.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract-prevention-risques_V1.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract-avenant-TL-v2.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_calculateur_salaires_2025.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/CGT-NPS-Voeux-2025.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract-indus-v1.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/2024-12-04_Mobilisations_et_elections_TPE.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_bilan_rcc24_v4.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_democratie_rcc_salaires_v2.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Profession_de_Foi_CGT_elections_FCPAN_2024_VF_V3.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_retour_salaires_2024_v1.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/reorg-mn-V3.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract-noel-2023-V3.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/ncc%20cotation%203.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_annonces_pekka_06_11_2023.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_militants_nord.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract%20com%20nokia%20final.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/midpoints.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Tract%20Volontariat%20RCC.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Tract%20br%C3%A8ves%20de%20printemps.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Tract_Sant%C3%A9_Pr%C3%A9voyance_Mars_2022%20nps.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Tract%20CGT%20desaccords%20en%20cascade%2003-06-2022.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Tract%20br%C3%A8ves%20d%27%C3%A9t%C3%A9.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Tract%20demenagement%2006-09-22.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Manif29septembre%20CandidaturesElection.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Ce%20que%20veulent%20les%20Cadres%20-Synth%C3%A8se%20Barom%C3%A8tre%20Cadres%20UGICT%20Viavoice%20octobre%202022.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Retour%20Sondage%20CGT%20Navettes%20Octobre%202022.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Les%20Navettes%20Quelle%20Gal%C3%A8re%2009_11_2022.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Radar%20Travail%20et%20Environnement%2009_11_2022.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Le%20saviez-vous%2012_11_2022.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Points%20sur%20les%20i%2012_11_2022.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Elections%20Pro%20-%20Choisir%20son%20camp.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Enjeu%20Salaires2022.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Tract%20Sondages.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Tract_NegoTELEW.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Bilans%20des%20accords%20sign%C3%A9s%20par%20la%20CGT.pdf</t>
   </si>
   <si>
     <t>Objet du courriel</t>
@@ -2852,8 +2852,8 @@
 </file>
 
 <file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005C9E45C7454FD54C9F3832CA2EC2299C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="598b0ce14474b8a06003600b576ad2b7">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xmlns:ns3="4a0c25b5-f40f-4aa1-8c63-969f2512d63e" xmlns:ns4="98344022-9d6c-42ca-8763-b68a110aeabc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f3517c15821bb310180c621d8d765fa" ns2:_="" ns3:_="" ns4:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005C9E45C7454FD54C9F3832CA2EC2299C" ma:contentTypeVersion="18" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="f12b8f105f65fc626cd1ca7eb8beb4c8">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xmlns:ns3="4a0c25b5-f40f-4aa1-8c63-969f2512d63e" xmlns:ns4="98344022-9d6c-42ca-8763-b68a110aeabc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="982fd3aadd5e0000c6cf8d705096d1e3" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
     <xsd:import namespace="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
     <xsd:import namespace="98344022-9d6c-42ca-8763-b68a110aeabc"/>
@@ -2907,12 +2907,12 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="_dlc_DocId" ma:index="24" nillable="true" ma:displayName="Document ID Value" ma:description="The value of the document ID assigned to this item." ma:indexed="true" ma:internalName="_dlc_DocId" ma:readOnly="true">
+    <xsd:element name="_dlc_DocId" ma:index="24" nillable="true" ma:displayName="Valeur d’ID de document" ma:description="Valeur de l’ID de document affecté à cet élément." ma:indexed="true" ma:internalName="_dlc_DocId" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="_dlc_DocIdUrl" ma:index="25" nillable="true" ma:displayName="Document ID" ma:description="Permanent link to this document." ma:hidden="true" ma:internalName="_dlc_DocIdUrl" ma:readOnly="true">
+    <xsd:element name="_dlc_DocIdUrl" ma:index="25" nillable="true" ma:displayName="ID de document" ma:description="Lien permanent vers ce document." ma:hidden="true" ma:internalName="_dlc_DocIdUrl" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:URL">
@@ -2953,7 +2953,7 @@
         <xsd:restriction base="dms:Unknown"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="16" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="16" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Balises d’images" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -2996,7 +2996,7 @@
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="98344022-9d6c-42ca-8763-b68a110aeabc" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="11" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="11" nillable="true" ma:displayName="Partagé avec" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -3015,7 +3015,7 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="12" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="12" nillable="true" ma:displayName="Partagé avec détails" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
@@ -3032,8 +3032,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Type de contenu"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titre"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -3158,23 +3158,7 @@
 </file>
 
 <file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7240B62-D29F-4BAF-A962-8ED89B4B626A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
-    <ds:schemaRef ds:uri="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
-    <ds:schemaRef ds:uri="98344022-9d6c-42ca-8763-b68a110aeabc"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F886958-6714-4C6B-B8BA-2D30B483596D}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>